<commit_message>
fix: update partner type wording to include Commission Agent
</commit_message>
<xml_diff>
--- a/next_app/public/templates/contact_import_template.xlsx
+++ b/next_app/public/templates/contact_import_template.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Farmer (Producer)</t>
+          <t>Farmer</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Buyer (Trader)</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -588,7 +588,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Your entry is not in the list" promptTitle="Select Partner Type" prompt="Please select from the list" type="list">
-      <formula1>"Farmer (Producer),Buyer (Trader),External Supplier"</formula1>
+      <formula1>"Farmer,Buyer,Commission Agent"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Your entry is not in the list" promptTitle="Select Balance Type" prompt="Please select To Receive or To Pay" type="list">
       <formula1>"To Receive,To Pay"</formula1>

</xml_diff>

<commit_message>
chore: change Commission Agent to Supplier in Excel import template
</commit_message>
<xml_diff>
--- a/next_app/public/templates/contact_import_template.xlsx
+++ b/next_app/public/templates/contact_import_template.xlsx
@@ -1,47 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0010B981"/>
-        <bgColor rgb="0010B981"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,16 +41,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -212,6 +194,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -246,6 +229,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -280,20 +264,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -415,7 +395,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -428,66 +447,54 @@
   </sheetPr>
   <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Partner Type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Opening Balance</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Balance Type</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>GSTIN</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>PAN</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PIN Code</t>
         </is>
@@ -522,8 +529,6 @@
           <t>To Pay</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Maharashtra</t>
@@ -586,12 +591,9 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Your entry is not in the list" promptTitle="Select Partner Type" prompt="Please select from the list" type="list">
-      <formula1>"Farmer,Buyer,Commission Agent"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Your entry is not in the list" promptTitle="Select Balance Type" prompt="Please select To Receive or To Pay" type="list">
-      <formula1>"To Receive,To Pay"</formula1>
+      <formula1>"Farmer,Buyer,Supplier"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: add balance type data validation dropdown to contact import template
</commit_message>
<xml_diff>
--- a/next_app/public/templates/contact_import_template.xlsx
+++ b/next_app/public/templates/contact_import_template.xlsx
@@ -1,24 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,13 +49,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -194,7 +203,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -229,7 +237,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -264,16 +271,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -395,46 +406,7 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -445,155 +417,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Partner Type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Opening Balance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Balance Type</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>GSTIN</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PAN</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PIN Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ramesh Singh</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Farmer</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Nashik</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>To Pay</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Maharashtra</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>422001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>A1 Traders</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Buyer</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>9123456780</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>12000</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>To Receive</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>27AAAAA0000A1Z5</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>AAAAA0000A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Maharashtra</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>400001</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Your entry is not in the list" promptTitle="Select Partner Type" prompt="Please select from the list" type="list">
-      <formula1>"Farmer,Buyer,Supplier"</formula1>
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Buyer,Farmer,Supplier"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"To Pay,To Receive"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: add sample records to contact import template
</commit_message>
<xml_diff>
--- a/next_app/public/templates/contact_import_template.xlsx
+++ b/next_app/public/templates/contact_import_template.xlsx
@@ -29,12 +29,18 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E5E7EB"/>
+        <bgColor rgb="00E5E7EB"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -51,7 +57,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -484,6 +490,140 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ramesh Farmer</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Farmer</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nashik</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>To Pay</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>422001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ABC Traders</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Buyer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>9123456780</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>To Receive</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>27AAAAA0000A1Z5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>AAAAA0000A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>400001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>XYZ Suppliers</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>9988776655</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>To Pay</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>411001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>